<commit_message>
Add verified phone numbers and addresses; remove closed organizations
Researched and verified real contact info (phone + street address) for
every organization from official sources. Removed Refugee Services of
Texas-Houston and The Alliance for Multicultural Community Services,
both confirmed permanently closed. Corrected neighborhood/zip for a
few entries where the verified office address didn't match the prior
tag. Added address and "get directions" links to the web app cards,
and a visible flag on any listing still missing both phone and
website. Updated findings.md and README to reflect the corrected gap
analysis, which now shows Gulfton with no verified local presence in
four of five service categories.
</commit_message>
<xml_diff>
--- a/dashboard/Houston_Community_Resource_Dashboard.xlsx
+++ b/dashboard/Houston_Community_Resource_Dashboard.xlsx
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -710,7 +710,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -732,17 +732,25 @@
           <t>77023</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>713-929-2330</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>aama.org</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Free ESL adult basic education GED computer literacy and workforce certification classes plus free child care for qualifying students. Contact via 211texas.org.</t>
+          <t>Free ESL adult basic education GED computer literacy and workforce certification classes plus free child care for qualifying students.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -764,10 +772,14 @@
           <t>77009</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>713-869-1684</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>avance.org</t>
+          <t>avancehouston.org</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -778,7 +790,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -814,7 +826,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -832,7 +844,11 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>713-692-6216</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>hcde-texas.org</t>
@@ -846,7 +862,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -864,7 +880,11 @@
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>832-393-1313</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>houstonlibrary.org</t>
@@ -878,7 +898,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -897,10 +917,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>77043</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
+          <t>77080</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>713-468-4516</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>mamhouston.org</t>
@@ -914,7 +938,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -928,15 +952,19 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Northwest Houston</t>
+          <t>East Houston</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>77092</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>77029</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>713-223-3700</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>houstonfoodbank.org</t>
@@ -950,7 +978,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -964,12 +992,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Montrose</t>
+          <t>Downtown</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>77006</t>
+          <t>77002</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -990,7 +1018,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -1008,7 +1036,11 @@
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>713-695-5437</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>kidsmealsinc.org</t>
@@ -1022,7 +1054,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1044,7 +1076,11 @@
           <t>77026</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>713-226-4953</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>targethunger.org</t>
@@ -1058,7 +1094,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1080,8 +1116,16 @@
           <t>77011</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>713-660-1880</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>elcentrodecorazon.org</t>
+        </is>
+      </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Federally qualified health center serving low-income and predominantly Hispanic families in Houston's East End with medical and dental care.</t>
@@ -1090,7 +1134,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1112,8 +1156,16 @@
           <t>77036</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>713-773-0803</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>hopechc.org</t>
+        </is>
+      </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Multicultural community health center providing primary medical dental and behavioral health care for low-income and immigrant families.</t>
@@ -1122,7 +1174,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1140,7 +1192,11 @@
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>832-548-5000</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>legacycommunityhealth.org</t>
@@ -1154,7 +1210,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1173,10 +1229,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>77081</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>77074</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>713-273-3700</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>bakerripley.org</t>
@@ -1190,7 +1250,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1212,7 +1272,11 @@
           <t>77072</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>281-530-6888</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>bpsos.org</t>
@@ -1226,7 +1290,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1240,15 +1304,19 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Spring Branch</t>
+          <t>Sharpstown</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>77055</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>77074</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>346-200-9951</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>cwshouston.org</t>
@@ -1262,7 +1330,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1302,7 +1370,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1320,7 +1388,11 @@
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>979-255-5188</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>houstonwelcomesrefugees.com</t>
@@ -1338,7 +1410,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Refugee Services of Texas - Houston</t>
+          <t>USCRI Houston</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1353,24 +1425,28 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>77036</t>
+          <t>77082</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>refugees.org</t>
+        </is>
+      </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Resettlement support and case management for refugees asylees and survivors of trafficking from more than 30 countries of origin. Contact via 211texas.org for current details.</t>
+          <t>Field office of the U.S. Committee for Refugees and Immigrants providing integration support health navigation and partner referrals for newly arrived families.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>The Alliance for Multicultural Community Services</t>
+          <t>YMCA International Services</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1380,93 +1456,25 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Gulfton</t>
+          <t>Southwest Houston</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>77081</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
+          <t>77057</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>346-297-2373</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>ymcahouston.org</t>
+        </is>
+      </c>
       <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Three-decade-old agency helping refugees immigrants and low-income residents with cultural adjustment economic self-sufficiency and mental health support.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>USCRI Houston</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Refugee &amp; Immigration Services</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Southwest Houston</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>77036</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>refugees.org</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Field office of the U.S. Committee for Refugees and Immigrants providing integration support health navigation and partner referrals for newly arrived families.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>YMCA International Services</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Refugee &amp; Immigration Services</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Gulfton</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>77081</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>346-297-2373</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>ymcahouston.org</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Case management cultural orientation employment services and immigration legal help for refugees and immigrants in one of Houston's most diverse zip codes.</t>
         </is>
@@ -1546,23 +1554,23 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A4,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A4,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A4,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A4,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A4,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G4" s="6">
@@ -1577,23 +1585,23 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G5" s="6">
@@ -1608,23 +1616,23 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G6" s="6">
@@ -1639,23 +1647,23 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G7" s="6">
@@ -1666,27 +1674,27 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>East End</t>
+          <t>Downtown</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G8" s="6">
@@ -1697,27 +1705,27 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Midtown</t>
+          <t>East End</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G9" s="6">
@@ -1728,27 +1736,27 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Montrose</t>
+          <t>East Houston</t>
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G10" s="6">
@@ -1759,27 +1767,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Near Northside</t>
+          <t>Midtown</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G11" s="6">
@@ -1790,27 +1798,27 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Northside</t>
+          <t>Near Northside</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G12" s="6">
@@ -1821,27 +1829,27 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Northwest Houston</t>
+          <t>Northside</t>
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G13" s="6">
@@ -1856,23 +1864,23 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G14" s="6">
@@ -1887,23 +1895,23 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,B$3)</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,C$3)</f>
         <v/>
       </c>
       <c r="D15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,D$3)</f>
         <v/>
       </c>
       <c r="E15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,E$3)</f>
         <v/>
       </c>
       <c r="F15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,F$3)</f>
         <v/>
       </c>
       <c r="G15" s="6">
@@ -1988,7 +1996,7 @@
         </is>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A5,Resources!$C$2:$C$23,$B5)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,$B5)</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -2008,7 +2016,7 @@
         </is>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A6,Resources!$C$2:$C$23,$B6)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,$B6)</f>
         <v/>
       </c>
       <c r="D6" s="6">
@@ -2028,7 +2036,7 @@
         </is>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A7,Resources!$C$2:$C$23,$B7)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,$B7)</f>
         <v/>
       </c>
       <c r="D7" s="6">
@@ -2048,7 +2056,7 @@
         </is>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A8,Resources!$C$2:$C$23,$B8)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,$B8)</f>
         <v/>
       </c>
       <c r="D8" s="6">
@@ -2068,7 +2076,7 @@
         </is>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A9,Resources!$C$2:$C$23,$B9)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,$B9)</f>
         <v/>
       </c>
       <c r="D9" s="6">
@@ -2088,7 +2096,7 @@
         </is>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A10,Resources!$C$2:$C$23,$B10)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,$B10)</f>
         <v/>
       </c>
       <c r="D10" s="6">
@@ -2108,7 +2116,7 @@
         </is>
       </c>
       <c r="C11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A11,Resources!$C$2:$C$23,$B11)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,$B11)</f>
         <v/>
       </c>
       <c r="D11" s="6">
@@ -2128,7 +2136,7 @@
         </is>
       </c>
       <c r="C12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A12,Resources!$C$2:$C$23,$B12)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,$B12)</f>
         <v/>
       </c>
       <c r="D12" s="6">
@@ -2148,7 +2156,7 @@
         </is>
       </c>
       <c r="C13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A13,Resources!$C$2:$C$23,$B13)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,$B13)</f>
         <v/>
       </c>
       <c r="D13" s="6">
@@ -2168,7 +2176,7 @@
         </is>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A14,Resources!$C$2:$C$23,$B14)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,$B14)</f>
         <v/>
       </c>
       <c r="D14" s="6">
@@ -2188,7 +2196,7 @@
         </is>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A15,Resources!$C$2:$C$23,$B15)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,$B15)</f>
         <v/>
       </c>
       <c r="D15" s="6">
@@ -2208,7 +2216,7 @@
         </is>
       </c>
       <c r="C16" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A16,Resources!$C$2:$C$23,$B16)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A16,Resources!$C$2:$C$21,$B16)</f>
         <v/>
       </c>
       <c r="D16" s="6">
@@ -2228,7 +2236,7 @@
         </is>
       </c>
       <c r="C17" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A17,Resources!$C$2:$C$23,$B17)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A17,Resources!$C$2:$C$21,$B17)</f>
         <v/>
       </c>
       <c r="D17" s="6">
@@ -2248,7 +2256,7 @@
         </is>
       </c>
       <c r="C18" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A18,Resources!$C$2:$C$23,$B18)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A18,Resources!$C$2:$C$21,$B18)</f>
         <v/>
       </c>
       <c r="D18" s="6">
@@ -2268,7 +2276,7 @@
         </is>
       </c>
       <c r="C19" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A19,Resources!$C$2:$C$23,$B19)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A19,Resources!$C$2:$C$21,$B19)</f>
         <v/>
       </c>
       <c r="D19" s="6">
@@ -2288,7 +2296,7 @@
         </is>
       </c>
       <c r="C20" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A20,Resources!$C$2:$C$23,$B20)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A20,Resources!$C$2:$C$21,$B20)</f>
         <v/>
       </c>
       <c r="D20" s="6">
@@ -2308,7 +2316,7 @@
         </is>
       </c>
       <c r="C21" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A21,Resources!$C$2:$C$23,$B21)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A21,Resources!$C$2:$C$21,$B21)</f>
         <v/>
       </c>
       <c r="D21" s="6">
@@ -2328,7 +2336,7 @@
         </is>
       </c>
       <c r="C22" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A22,Resources!$C$2:$C$23,$B22)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A22,Resources!$C$2:$C$21,$B22)</f>
         <v/>
       </c>
       <c r="D22" s="6">
@@ -2348,7 +2356,7 @@
         </is>
       </c>
       <c r="C23" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A23,Resources!$C$2:$C$23,$B23)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A23,Resources!$C$2:$C$21,$B23)</f>
         <v/>
       </c>
       <c r="D23" s="6">
@@ -2368,7 +2376,7 @@
         </is>
       </c>
       <c r="C24" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$23,$A24,Resources!$C$2:$C$23,$B24)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$21,$A24,Resources!$C$2:$C$21,$B24)</f>
         <v/>
       </c>
       <c r="D24" s="6">

</xml_diff>

<commit_message>
Add Farsi/Vietnamese support and Clothing & Household Goods category
Adds two more languages to the toggle (Farsi with full right-to-left
layout, Vietnamese), covering the Afghan/Persian-speaking and
Vietnamese communities this project's own neighborhood data documents
in Gulfton and Alief. Every UI string, organization description, and
neighborhood profile is translated in both, not just labels.

Also adds a sixth resource category, Clothing & Household Goods,
with 7 verified organizations (church clothes closets, a Catholic
Worker house, a furniture bank, emergency clothing centers) found
through research and checked against official sources. Several
candidates were investigated and left out because they turned out to
be closed or unverifiable, documented in findings.md. The new
category updates the gap analysis: Gulfton, Alief, and Sharpstown
still have no verified local presence in it, while Spring Branch has
two.
</commit_message>
<xml_diff>
--- a/dashboard/Houston_Community_Resource_Dashboard.xlsx
+++ b/dashboard/Houston_Community_Resource_Dashboard.xlsx
@@ -262,12 +262,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$A$4:$A$15</f>
+              <f>'Summary'!$A$4:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$G$4:$G$15</f>
+              <f>'Summary'!$G$4:$G$20</f>
             </numRef>
           </val>
         </ser>
@@ -343,7 +343,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3240000"/>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -710,712 +710,720 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>AAMA Adelante Adult Literacy</t>
+          <t>Casa Juan Diego</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>East End</t>
+          <t>Houston Heights</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>77023</t>
+          <t>77007</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>713-929-2330</t>
+          <t>713-869-7376</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>aama.org</t>
+          <t>cjd.org</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Free ESL adult basic education GED computer literacy and workforce certification classes plus free child care for qualifying students.</t>
+          <t>Catholic Worker house of hospitality offering weekly free food and clothing distribution plus household-goods assistance specifically for immigrant and refugee families.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AVANCE-Houston</t>
+          <t>Christian Community Service Center - Emergency Services Central</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Northside</t>
+          <t>Greenway</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>77009</t>
+          <t>77027</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>713-869-1684</t>
+          <t>713-871-9741</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>avancehouston.org</t>
+          <t>ccschouston.org</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Parent and early-childhood education programs including ESL Head Start and General Equivalency Diploma preparation for low-income families.</t>
+          <t>This Emergency Services Central location provides gently used clothing diapers hygiene kits and a five-day food package after a walk-in interview; CCSC's Southwest branch offers food and hygiene only not clothing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BakerRipley Adult Education</t>
+          <t>Emergency Aid Coalition - Clothing Center</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>Third Ward</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>77004</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>713-273-3719</t>
+          <t>713-343-3061</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>economicinitiatives.bakerripley.org</t>
+          <t>eachouston.org</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Free ESL GED and computer literacy classes for adult learners at multiple campuses across Harris County with no minimum education requirement.</t>
+          <t>Free clothing up to two outfits per person shoes when available toiletries and underwear for men women and children with visits by appointment only.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HCDE Adult Education ESL</t>
+          <t>Faith Center Spring Branch</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>Spring Branch</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>77055</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>713-692-6216</t>
+          <t>713-554-8820</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>hcde-texas.org</t>
+          <t>houstonsfirst.org</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Harris County Department of Education program offering free beginning through advanced ESL classes online and in person across the county.</t>
+          <t>Free food pantry and clothes closet providing groceries clothing and hygiene essentials to Spring Branch families with visits by appointment.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Houston Public Library - Cultural Connections &amp; ESL</t>
+          <t>Houston Furniture Bank</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>South Houston</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>77075</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>832-393-1313</t>
+          <t>713-842-9777</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>houstonlibrary.org</t>
+          <t>houstonfurniturebank.org</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Free English and language-learning classes plus cultural-orientation programming open to new immigrants at branches across the city.</t>
+          <t>Provides free furniture such as beds tables seating and mattresses to families in need but only through referral from a partner social-service agency not direct walk-in.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Literacy Advance - Memorial Assistance Ministries</t>
+          <t>Lilly Grove Missionary Baptist Church - Clothes Closet</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Education &amp; ESL</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Spring Branch</t>
+          <t>South Union</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>77080</t>
+          <t>77021</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>713-468-4516</t>
+          <t>713-748-7324</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>mamhouston.org</t>
+          <t>lillygrove.org</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Free English and reading classes for adults running since 1964 supported by volunteer tutors plus citizenship and employment-readiness classes.</t>
+          <t>Free clothing for men women and children including suits shirts casual wear shoes undergarments uniforms and backpacks from a dedicated house across from the church.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Houston Food Bank</t>
+          <t>Memorial Assistance Ministries - Resale &amp; Voucher Program</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Food Assistance</t>
+          <t>Clothing &amp; Household Goods</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>East Houston</t>
+          <t>Spring Branch</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>77029</t>
+          <t>77080</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>713-223-3700</t>
+          <t>713-491-4330</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>houstonfoodbank.org</t>
+          <t>mamhouston.org</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Largest hunger-relief organization in southeast Texas coordinating pantries meal programs and produce distributions across 18 counties.</t>
+          <t>Issues clothing and furniture vouchers redeemable at the MAM Resale Store which also sells low-cost clothing home furnishings electronics and household items.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Interfaith Ministries for Greater Houston</t>
+          <t>AAMA Adelante Adult Literacy</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Food Assistance</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Downtown</t>
+          <t>East End</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>77002</t>
+          <t>77023</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>713-533-4900</t>
+          <t>713-929-2330</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>imgh.org</t>
+          <t>aama.org</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Emergency food assistance and a Meals on Wheels senior meals program alongside refugee housing English classes and job placement support.</t>
+          <t>Free ESL adult basic education GED computer literacy and workforce certification classes plus free child care for qualifying students.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kids' Meals</t>
+          <t>AVANCE-Houston</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Food Assistance</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>Northside</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>77009</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>713-695-5437</t>
+          <t>713-869-1684</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>kidsmealsinc.org</t>
+          <t>avancehouston.org</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Delivers free healthy meals on weekdays to the homes of children under six and connects families to a broader support network.</t>
+          <t>Parent and early-childhood education programs including ESL Head Start and General Equivalency Diploma preparation for low-income families.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Target Hunger</t>
+          <t>BakerRipley Adult Education</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Food Assistance</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Near Northside</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>77026</t>
-        </is>
-      </c>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>713-226-4953</t>
+          <t>713-273-3719</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>targethunger.org</t>
+          <t>economicinitiatives.bakerripley.org</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Food assistance and navigation programs that provided food to more than 25000 individuals and 9200 households across Houston in 2025.</t>
+          <t>Free ESL GED and computer literacy classes for adult learners at multiple campuses across Harris County with no minimum education requirement.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>El Centro de Corazon</t>
+          <t>HCDE Adult Education ESL</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>East End</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>77011</t>
-        </is>
-      </c>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>713-660-1880</t>
+          <t>713-692-6216</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>elcentrodecorazon.org</t>
+          <t>hcde-texas.org</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Federally qualified health center serving low-income and predominantly Hispanic families in Houston's East End with medical and dental care.</t>
+          <t>Harris County Department of Education program offering free beginning through advanced ESL classes online and in person across the county.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HOPE Clinic</t>
+          <t>Houston Public Library - Cultural Connections &amp; ESL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Southwest Houston</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>77036</t>
-        </is>
-      </c>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>713-773-0803</t>
+          <t>832-393-1313</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>hopechc.org</t>
+          <t>houstonlibrary.org</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Multicultural community health center providing primary medical dental and behavioral health care for low-income and immigrant families.</t>
+          <t>Free English and language-learning classes plus cultural-orientation programming open to new immigrants at branches across the city.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Legacy Community Health</t>
+          <t>Literacy Advance - Memorial Assistance Ministries</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Education &amp; ESL</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>Spring Branch</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>77080</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>832-548-5000</t>
+          <t>713-468-4516</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>legacycommunityhealth.org</t>
+          <t>mamhouston.org</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Federally qualified health network with clinics across Houston offering sliding-scale primary care for low-income and uninsured residents.</t>
+          <t>Free English and reading classes for adults running since 1964 supported by volunteer tutors plus citizenship and employment-readiness classes.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>BakerRipley Gulfton-Sharpstown Campus</t>
+          <t>Houston Food Bank</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Multi-Service Community Center</t>
+          <t>Food Assistance</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Gulfton</t>
+          <t>East Houston</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>77074</t>
+          <t>77029</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>713-273-3700</t>
+          <t>713-223-3700</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>bakerripley.org</t>
+          <t>houstonfoodbank.org</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Five-building neighborhood campus offering early childhood education youth programs immigration services and a community garden for residents from 80-plus countries.</t>
+          <t>Largest hunger-relief organization in southeast Texas coordinating pantries meal programs and produce distributions across 18 counties.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>BPSOS-Houston</t>
+          <t>Interfaith Ministries for Greater Houston</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Refugee &amp; Immigration Services</t>
+          <t>Food Assistance</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Alief</t>
+          <t>Downtown</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>77072</t>
+          <t>77002</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>281-530-6888</t>
+          <t>713-533-4900</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>bpsos.org</t>
+          <t>imgh.org</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Boat People S.O.S. affiliate supporting Vietnamese and other Southeast Asian immigrant and refugee families with case management and civic engagement.</t>
+          <t>Emergency food assistance and a Meals on Wheels senior meals program alongside refugee housing English classes and job placement support.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CWS Houston</t>
+          <t>Kids' Meals</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Refugee &amp; Immigration Services</t>
+          <t>Food Assistance</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Sharpstown</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>77074</t>
-        </is>
-      </c>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>346-200-9951</t>
+          <t>713-695-5437</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>cwshouston.org</t>
+          <t>kidsmealsinc.org</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Resettlement case management housing assistance ESL and cultural orientation referrals and support for unaccompanied minors transitioning into local care.</t>
+          <t>Delivers free healthy meals on weekdays to the homes of children under six and connects families to a broader support network.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Catholic Charities of the Archdiocese of Galveston-Houston</t>
+          <t>Target Hunger</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Refugee &amp; Immigration Services</t>
+          <t>Food Assistance</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Midtown</t>
+          <t>Near Northside</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>77006</t>
+          <t>77026</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>713-526-4611</t>
+          <t>713-226-4953</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>catholiccharities.org</t>
+          <t>targethunger.org</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Refugee resettlement immigration legal services family strengthening and senior services serving more than 85000 people a year across the region.</t>
+          <t>Food assistance and navigation programs that provided food to more than 25000 individuals and 9200 households across Houston in 2025.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Houston Welcomes Refugees</t>
+          <t>El Centro de Corazon</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Refugee &amp; Immigration Services</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Citywide</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>East End</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>77011</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>979-255-5188</t>
+          <t>713-660-1880</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>houstonwelcomesrefugees.com</t>
+          <t>elcentrodecorazon.org</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Volunteer welcome teams that deliver welcome kits and groceries and connect newly arrived refugees to critical resources in their first months.</t>
+          <t>Federally qualified health center serving low-income and predominantly Hispanic families in Houston's East End with medical and dental care.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>USCRI Houston</t>
+          <t>HOPE Clinic</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Refugee &amp; Immigration Services</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1425,56 +1433,328 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>77082</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>77036</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>713-773-0803</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>refugees.org</t>
+          <t>hopechc.org</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Field office of the U.S. Committee for Refugees and Immigrants providing integration support health navigation and partner referrals for newly arrived families.</t>
+          <t>Multicultural community health center providing primary medical dental and behavioral health care for low-income and immigrant families.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Community Health</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>832-548-5000</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>legacycommunityhealth.org</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Federally qualified health network with clinics across Houston offering sliding-scale primary care for low-income and uninsured residents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>BakerRipley Gulfton-Sharpstown Campus</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Multi-Service Community Center</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Gulfton</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>77074</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>713-273-3700</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>bakerripley.org</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Five-building neighborhood campus offering early childhood education youth programs immigration services and a community garden for residents from 80-plus countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>BPSOS-Houston</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Refugee &amp; Immigration Services</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Alief</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>77072</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>281-530-6888</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>bpsos.org</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Boat People S.O.S. affiliate supporting Vietnamese and other Southeast Asian immigrant and refugee families with case management and civic engagement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>CWS Houston</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Refugee &amp; Immigration Services</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Sharpstown</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>77074</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>346-200-9951</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>cwshouston.org</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Resettlement case management housing assistance ESL and cultural orientation referrals and support for unaccompanied minors transitioning into local care.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Catholic Charities of the Archdiocese of Galveston-Houston</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Refugee &amp; Immigration Services</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Midtown</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>77006</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>713-526-4611</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>catholiccharities.org</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Refugee resettlement immigration legal services family strengthening and senior services serving more than 85000 people a year across the region.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Houston Welcomes Refugees</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Refugee &amp; Immigration Services</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>979-255-5188</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>houstonwelcomesrefugees.com</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Volunteer welcome teams that deliver welcome kits and groceries and connect newly arrived refugees to critical resources in their first months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>USCRI Houston</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Refugee &amp; Immigration Services</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Southwest Houston</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>77082</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>refugees.org</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Field office of the U.S. Committee for Refugees and Immigrants providing integration support health navigation and partner referrals for newly arrived families.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>YMCA International Services</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Refugee &amp; Immigration Services</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Southwest Houston</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>77057</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>346-297-2373</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>ymcahouston.org</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Case management cultural orientation employment services and immigration legal help for refugees and immigrants in one of Houston's most diverse zip codes.</t>
         </is>
@@ -1491,7 +1771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1554,23 +1834,23 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A4,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A4,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A4,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A4,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F4" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A4,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A4,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G4" s="6">
@@ -1585,23 +1865,23 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G5" s="6">
@@ -1616,23 +1896,23 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G6" s="6">
@@ -1647,23 +1927,23 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G7" s="6">
@@ -1678,23 +1958,23 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G8" s="6">
@@ -1709,23 +1989,23 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G9" s="6">
@@ -1740,23 +2020,23 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G10" s="6">
@@ -1767,27 +2047,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Midtown</t>
+          <t>Greenway</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G11" s="6">
@@ -1798,27 +2078,27 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Near Northside</t>
+          <t>Houston Heights</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G12" s="6">
@@ -1829,27 +2109,27 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Northside</t>
+          <t>Midtown</t>
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G13" s="6">
@@ -1860,27 +2140,27 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Southwest Houston</t>
+          <t>Near Northside</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G14" s="6">
@@ -1891,31 +2171,186 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Citywide</t>
+          <t>Northside</t>
         </is>
       </c>
       <c r="B15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,B$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,B$3)</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,C$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,C$3)</f>
         <v/>
       </c>
       <c r="D15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,D$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,D$3)</f>
         <v/>
       </c>
       <c r="E15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,E$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,E$3)</f>
         <v/>
       </c>
       <c r="F15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,F$3)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,F$3)</f>
         <v/>
       </c>
       <c r="G15" s="6">
         <f>SUM(B15:F15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>South Houston</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,B$3)</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,C$3)</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,D$3)</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,E$3)</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,F$3)</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>South Union</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,B$3)</f>
+        <v/>
+      </c>
+      <c r="C17" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,C$3)</f>
+        <v/>
+      </c>
+      <c r="D17" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,D$3)</f>
+        <v/>
+      </c>
+      <c r="E17" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,E$3)</f>
+        <v/>
+      </c>
+      <c r="F17" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,F$3)</f>
+        <v/>
+      </c>
+      <c r="G17" s="6">
+        <f>SUM(B17:F17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Southwest Houston</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,B$3)</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,C$3)</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,D$3)</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,E$3)</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,F$3)</f>
+        <v/>
+      </c>
+      <c r="G18" s="6">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Third Ward</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,B$3)</f>
+        <v/>
+      </c>
+      <c r="C19" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,C$3)</f>
+        <v/>
+      </c>
+      <c r="D19" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,D$3)</f>
+        <v/>
+      </c>
+      <c r="E19" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,E$3)</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,F$3)</f>
+        <v/>
+      </c>
+      <c r="G19" s="6">
+        <f>SUM(B19:F19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Citywide</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,B$3)</f>
+        <v/>
+      </c>
+      <c r="C20" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,C$3)</f>
+        <v/>
+      </c>
+      <c r="D20" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,D$3)</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,E$3)</f>
+        <v/>
+      </c>
+      <c r="F20" s="6">
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,F$3)</f>
+        <v/>
+      </c>
+      <c r="G20" s="6">
+        <f>SUM(B20:F20)</f>
         <v/>
       </c>
     </row>
@@ -1923,7 +2358,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:F15">
+  <conditionalFormatting sqref="B4:F20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1996,7 +2431,7 @@
         </is>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A5,Resources!$C$2:$C$21,$B5)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A5,Resources!$C$2:$C$28,$B5)</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -2016,7 +2451,7 @@
         </is>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A6,Resources!$C$2:$C$21,$B6)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A6,Resources!$C$2:$C$28,$B6)</f>
         <v/>
       </c>
       <c r="D6" s="6">
@@ -2036,7 +2471,7 @@
         </is>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A7,Resources!$C$2:$C$21,$B7)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A7,Resources!$C$2:$C$28,$B7)</f>
         <v/>
       </c>
       <c r="D7" s="6">
@@ -2056,7 +2491,7 @@
         </is>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A8,Resources!$C$2:$C$21,$B8)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A8,Resources!$C$2:$C$28,$B8)</f>
         <v/>
       </c>
       <c r="D8" s="6">
@@ -2076,7 +2511,7 @@
         </is>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A9,Resources!$C$2:$C$21,$B9)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A9,Resources!$C$2:$C$28,$B9)</f>
         <v/>
       </c>
       <c r="D9" s="6">
@@ -2096,7 +2531,7 @@
         </is>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A10,Resources!$C$2:$C$21,$B10)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A10,Resources!$C$2:$C$28,$B10)</f>
         <v/>
       </c>
       <c r="D10" s="6">
@@ -2116,7 +2551,7 @@
         </is>
       </c>
       <c r="C11" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A11,Resources!$C$2:$C$21,$B11)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A11,Resources!$C$2:$C$28,$B11)</f>
         <v/>
       </c>
       <c r="D11" s="6">
@@ -2136,7 +2571,7 @@
         </is>
       </c>
       <c r="C12" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A12,Resources!$C$2:$C$21,$B12)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A12,Resources!$C$2:$C$28,$B12)</f>
         <v/>
       </c>
       <c r="D12" s="6">
@@ -2156,7 +2591,7 @@
         </is>
       </c>
       <c r="C13" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A13,Resources!$C$2:$C$21,$B13)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A13,Resources!$C$2:$C$28,$B13)</f>
         <v/>
       </c>
       <c r="D13" s="6">
@@ -2176,7 +2611,7 @@
         </is>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A14,Resources!$C$2:$C$21,$B14)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A14,Resources!$C$2:$C$28,$B14)</f>
         <v/>
       </c>
       <c r="D14" s="6">
@@ -2196,7 +2631,7 @@
         </is>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A15,Resources!$C$2:$C$21,$B15)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A15,Resources!$C$2:$C$28,$B15)</f>
         <v/>
       </c>
       <c r="D15" s="6">
@@ -2216,7 +2651,7 @@
         </is>
       </c>
       <c r="C16" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A16,Resources!$C$2:$C$21,$B16)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A16,Resources!$C$2:$C$28,$B16)</f>
         <v/>
       </c>
       <c r="D16" s="6">
@@ -2236,7 +2671,7 @@
         </is>
       </c>
       <c r="C17" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A17,Resources!$C$2:$C$21,$B17)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A17,Resources!$C$2:$C$28,$B17)</f>
         <v/>
       </c>
       <c r="D17" s="6">
@@ -2256,7 +2691,7 @@
         </is>
       </c>
       <c r="C18" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A18,Resources!$C$2:$C$21,$B18)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A18,Resources!$C$2:$C$28,$B18)</f>
         <v/>
       </c>
       <c r="D18" s="6">
@@ -2276,7 +2711,7 @@
         </is>
       </c>
       <c r="C19" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A19,Resources!$C$2:$C$21,$B19)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A19,Resources!$C$2:$C$28,$B19)</f>
         <v/>
       </c>
       <c r="D19" s="6">
@@ -2296,7 +2731,7 @@
         </is>
       </c>
       <c r="C20" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A20,Resources!$C$2:$C$21,$B20)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A20,Resources!$C$2:$C$28,$B20)</f>
         <v/>
       </c>
       <c r="D20" s="6">
@@ -2316,7 +2751,7 @@
         </is>
       </c>
       <c r="C21" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A21,Resources!$C$2:$C$21,$B21)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A21,Resources!$C$2:$C$28,$B21)</f>
         <v/>
       </c>
       <c r="D21" s="6">
@@ -2336,7 +2771,7 @@
         </is>
       </c>
       <c r="C22" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A22,Resources!$C$2:$C$21,$B22)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A22,Resources!$C$2:$C$28,$B22)</f>
         <v/>
       </c>
       <c r="D22" s="6">
@@ -2356,7 +2791,7 @@
         </is>
       </c>
       <c r="C23" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A23,Resources!$C$2:$C$21,$B23)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A23,Resources!$C$2:$C$28,$B23)</f>
         <v/>
       </c>
       <c r="D23" s="6">
@@ -2376,7 +2811,7 @@
         </is>
       </c>
       <c r="C24" s="6">
-        <f>COUNTIFS(Resources!$D$2:$D$21,$A24,Resources!$C$2:$C$21,$B24)</f>
+        <f>COUNTIFS(Resources!$D$2:$D$28,$A24,Resources!$C$2:$C$28,$B24)</f>
         <v/>
       </c>
       <c r="D24" s="6">

</xml_diff>